<commit_message>
Fix dashboard text and polish workbook
</commit_message>
<xml_diff>
--- a/Medal_Forecasting_Portfolio_Synthetic.xlsx
+++ b/Medal_Forecasting_Portfolio_Synthetic.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{E264028B-B3A9-41DA-A7CF-F223D2601DED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2398548A-035A-4437-8CEC-75B05A255475}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{E264028B-B3A9-41DA-A7CF-F223D2601DED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46C5B328-5332-4031-8A8F-2DE0E6EA28E8}"/>
   <bookViews>
-    <workbookView xWindow="2004" yWindow="1896" windowWidth="20784" windowHeight="11412" tabRatio="880" activeTab="7" xr2:uid="{1F09CBC7-8482-8747-9E8F-75B3DA03EC9D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="880" activeTab="7" xr2:uid="{1F09CBC7-8482-8747-9E8F-75B3DA03EC9D}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="13" r:id="rId1"/>
@@ -333,9 +333,6 @@
     <t>2027 PURCHASING RECOMMENDATION</t>
   </si>
   <si>
-    <t>Preliminary estimates basedon on historical demand and forecasting errors. Update purchasing recommendations after 2026 actual demand, inventory reconciliaition, and vendor pricing are confirmed.</t>
-  </si>
-  <si>
     <t>Forecast Assumptions &amp; Methodology</t>
   </si>
   <si>
@@ -358,9 +355,6 @@
   </si>
   <si>
     <t>Greater of baseline buffer or maximum historical underforecast</t>
-  </si>
-  <si>
-    <t>2027 purchasing quantities are preliminary. Recalculate after 2026 actual demand, inventory reconciliation, and updated vendor pricing becomes available. Shipping estimates are based on prior years order.</t>
   </si>
   <si>
     <t>2026 demand and ending inventory are prelimary projections. Actual results will replace these estimates after the contest and inventory reconciliation.</t>
@@ -544,6 +538,12 @@
   <si>
     <t>$3.00 per medal</t>
   </si>
+  <si>
+    <t>Preliminary estimates based on historical demand and forecasting errors. Update purchasing recommendations after 2026 actual demand, inventory reconciliation, and vendor pricing are confirmed.</t>
+  </si>
+  <si>
+    <t>2027 purchasing quantities are preliminary. Recalculate after 2026 actual demand, inventory reconciliation, and updated vendor pricing becomes available. Shipping estimates are based on prior-years order.</t>
+  </si>
 </sst>
 </file>
 
@@ -551,7 +551,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
   <fonts count="29" x14ac:knownFonts="1">
     <font>
@@ -1034,7 +1034,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1251,10 +1251,10 @@
     <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="21" fillId="4" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1346,8 +1346,8 @@
     </xf>
     <xf numFmtId="1" fontId="18" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1391,10 +1391,45 @@
   </cellStyles>
   <dxfs count="24">
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1436,41 +1471,6 @@
           <bgColor theme="2" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -5902,17 +5902,17 @@
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{ECA31630-F135-48F5-A710-9B7FFCE5321F}" name="Classification"/>
     <tableColumn id="2" xr3:uid="{C5F191EF-21C9-44C9-986C-6B1B818A65BA}" name="Medal Type"/>
-    <tableColumn id="3" xr3:uid="{8E4750F6-699D-4B0F-AC8E-31203096B518}" name="2016" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{2BC00BD6-6D7E-4C89-BB06-FF542C2DAF44}" name="2017" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{294CD313-1754-4CD9-AE72-1F6E04C71309}" name="2018" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{EAFE8E2C-7BF8-4ABD-99DB-1063C5F8678E}" name="2019" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{5F434BD1-A2E9-414B-9E11-3A485EC5A1F9}" name="2020" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{2298156C-5554-4CBF-8537-05CA2EA38C14}" name="2021" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{262A32E4-5716-479A-A88C-FD6668396F7C}" name="2022" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{9E622BCB-9246-41DD-86DF-4C5B95A54309}" name="2023" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{E072A28B-986E-4277-B073-5C5592D29DE0}" name="2024" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{FB07C408-3F33-427C-B200-7264328E5B77}" name="2025" dataDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{01E15507-F1BA-43A8-9CC4-974536FD8924}" name="2026" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{8E4750F6-699D-4B0F-AC8E-31203096B518}" name="2016" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{2BC00BD6-6D7E-4C89-BB06-FF542C2DAF44}" name="2017" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{294CD313-1754-4CD9-AE72-1F6E04C71309}" name="2018" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{EAFE8E2C-7BF8-4ABD-99DB-1063C5F8678E}" name="2019" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{5F434BD1-A2E9-414B-9E11-3A485EC5A1F9}" name="2020" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{2298156C-5554-4CBF-8537-05CA2EA38C14}" name="2021" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{262A32E4-5716-479A-A88C-FD6668396F7C}" name="2022" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{9E622BCB-9246-41DD-86DF-4C5B95A54309}" name="2023" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{E072A28B-986E-4277-B073-5C5592D29DE0}" name="2024" dataDxfId="12"/>
+    <tableColumn id="12" xr3:uid="{FB07C408-3F33-427C-B200-7264328E5B77}" name="2025" dataDxfId="11"/>
+    <tableColumn id="13" xr3:uid="{01E15507-F1BA-43A8-9CC4-974536FD8924}" name="2026" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5925,8 +5925,8 @@
     <tableColumn id="1" xr3:uid="{2894D031-29CF-4D6B-800C-BEC386C37E4E}" name="Division"/>
     <tableColumn id="2" xr3:uid="{FDD5FD71-62A4-46D7-9E0D-F1E91D4E420B}" name="Forecasting Model"/>
     <tableColumn id="3" xr3:uid="{14B2C1B8-C5F9-459E-82C3-B05319180E3D}" name="MAE"/>
-    <tableColumn id="4" xr3:uid="{6CE26A0E-3647-4776-B7EF-DDEBB74309AC}" name="MAPE" dataDxfId="19" dataCellStyle="Percent"/>
-    <tableColumn id="5" xr3:uid="{B6C8B691-F4AB-4DE5-8218-6F30F3CB618C}" name="Bias" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{6CE26A0E-3647-4776-B7EF-DDEBB74309AC}" name="MAPE" dataDxfId="9" dataCellStyle="Percent"/>
+    <tableColumn id="5" xr3:uid="{B6C8B691-F4AB-4DE5-8218-6F30F3CB618C}" name="Bias" dataDxfId="8"/>
     <tableColumn id="6" xr3:uid="{A23D5F99-7597-4F88-8F78-354211565552}" name="2026 Forecast"/>
     <tableColumn id="7" xr3:uid="{F8DD691C-5A54-49D6-9227-1F7FF8DD51B8}" name="Best Model?">
       <calculatedColumnFormula>IF(C2=_xlfn.MINIFS($C$2:$C$10, $A$2:$A$10,A2), "Best","")</calculatedColumnFormula>
@@ -5941,10 +5941,10 @@
   <autoFilter ref="I1:K4" xr:uid="{5680078E-ACD3-4E11-854E-06BDF29B0561}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{1DB69119-707C-4086-AB0D-18E113A1F6A6}" name="Division"/>
-    <tableColumn id="2" xr3:uid="{B32B4845-1A1B-4C4C-B2D9-864304383730}" name="2026 Forecast" dataDxfId="17">
+    <tableColumn id="2" xr3:uid="{B32B4845-1A1B-4C4C-B2D9-864304383730}" name="2026 Forecast" dataDxfId="7">
       <calculatedColumnFormula>SUMIFS($F$2:$F$10, $A$2:$A$10, I2,$G$2:$G$10,"Best")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{1FF4C72D-0962-472B-AD31-80AAF7BDFD12}" name="2027 Forecast" dataDxfId="16">
+    <tableColumn id="3" xr3:uid="{1FF4C72D-0962-472B-AD31-80AAF7BDFD12}" name="2027 Forecast" dataDxfId="6">
       <calculatedColumnFormula>'1st Division'!L15</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5958,13 +5958,13 @@
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{5211E03E-5E99-4C3B-89B1-AF34B5E121DC}" name="Year"/>
     <tableColumn id="2" xr3:uid="{BE8F6832-4B10-4BAF-AC09-750F0527A577}" name="Division"/>
-    <tableColumn id="3" xr3:uid="{6D0866D2-CE56-4A93-8FCE-80715A3A5396}" name="Beginning Inventory" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{96B8447C-C777-4C65-A593-51D0067D6ACD}" name="Medals Purchased" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{6D0866D2-CE56-4A93-8FCE-80715A3A5396}" name="Beginning Inventory" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{96B8447C-C777-4C65-A593-51D0067D6ACD}" name="Medals Purchased" dataDxfId="4"/>
     <tableColumn id="5" xr3:uid="{EB4AC5FA-D76D-459C-B546-FFFAC2A71893}" name="Medals Awarded">
       <calculatedColumnFormula>SUMIF(Table1[Medal Type],B2,INDEX(Table1[],0,MATCH(A2&amp;"",Table1[#Headers],0)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{129B1229-E345-4F16-BFFE-6555F2BF3460}" name="Ending Inventory" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{915C2943-E8B0-4B11-8AD5-F53BA472D570}" name="Inventory Adjustment" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{129B1229-E345-4F16-BFFE-6555F2BF3460}" name="Ending Inventory" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{915C2943-E8B0-4B11-8AD5-F53BA472D570}" name="Inventory Adjustment" dataDxfId="2">
       <calculatedColumnFormula>F2-(C2+D2-E2)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{6370A42A-86BC-42A4-B832-D6E9A3695B0D}" name="Forecast Demand"/>
@@ -5988,7 +5988,7 @@
   <autoFilter ref="A1:B4" xr:uid="{4A42D987-28D3-438E-88FB-8723FA1F5E90}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{207139D5-E5D6-4C14-8E6A-852C28A3300B}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{D146D234-7859-49D3-A131-22F75715D89E}" name="Value" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{D146D234-7859-49D3-A131-22F75715D89E}" name="Value" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6300,7 +6300,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="46" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
@@ -6318,13 +6318,13 @@
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="41" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B3" s="41"/>
     </row>
     <row r="4" spans="1:6" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="39" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B4" s="39"/>
       <c r="C4" s="39"/>
@@ -6334,13 +6334,13 @@
     </row>
     <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="41" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B6" s="41"/>
     </row>
     <row r="7" spans="1:6" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="39" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B7" s="39"/>
       <c r="C7" s="39"/>
@@ -6350,13 +6350,13 @@
     </row>
     <row r="9" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="41" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B9" s="41"/>
     </row>
     <row r="10" spans="1:6" ht="127.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="47" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B10" s="47"/>
       <c r="C10" s="47"/>
@@ -6366,13 +6366,13 @@
     </row>
     <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="41" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B12" s="41"/>
     </row>
     <row r="13" spans="1:6" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="39" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B13" s="39"/>
       <c r="C13" s="39"/>
@@ -6385,10 +6385,10 @@
         <v>37</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C15" s="35" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -6399,7 +6399,7 @@
         <v>20</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -6410,7 +6410,7 @@
         <v>20</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -6421,7 +6421,7 @@
         <v>47</v>
       </c>
       <c r="C18" s="38" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -6429,12 +6429,12 @@
     </row>
     <row r="20" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A20" s="37" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="161.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="45" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B21" s="45"/>
       <c r="C21" s="45"/>
@@ -6444,13 +6444,13 @@
     </row>
     <row r="23" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A23" s="41" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B23" s="41"/>
     </row>
     <row r="24" spans="1:6" ht="145.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="39" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B24" s="39"/>
       <c r="C24" s="39"/>
@@ -6460,20 +6460,20 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="35" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B26" s="43" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C26" s="43"/>
       <c r="D26" s="43"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="38" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B27" s="42" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C27" s="42"/>
       <c r="D27" s="42"/>
@@ -6483,7 +6483,7 @@
         <v>92</v>
       </c>
       <c r="B28" s="42" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C28" s="42"/>
       <c r="D28" s="42"/>
@@ -6493,7 +6493,7 @@
         <v>70</v>
       </c>
       <c r="B29" s="42" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C29" s="42"/>
       <c r="D29" s="42"/>
@@ -6503,20 +6503,20 @@
         <v>64</v>
       </c>
       <c r="B30" s="42" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C30" s="42"/>
       <c r="D30" s="42"/>
     </row>
     <row r="32" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A32" s="44" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B32" s="44"/>
     </row>
     <row r="33" spans="1:12" ht="163.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="39" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B33" s="39"/>
       <c r="C33" s="39"/>
@@ -6526,13 +6526,13 @@
     </row>
     <row r="35" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A35" s="41" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B35" s="41"/>
     </row>
     <row r="36" spans="1:12" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="39" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B36" s="39"/>
       <c r="C36" s="39"/>
@@ -6542,13 +6542,13 @@
     </row>
     <row r="38" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A38" s="41" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B38" s="41"/>
     </row>
     <row r="39" spans="1:12" ht="162.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="39" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B39" s="39"/>
       <c r="C39" s="39"/>
@@ -6558,13 +6558,13 @@
     </row>
     <row r="41" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A41" s="41" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B41" s="41"/>
     </row>
     <row r="42" spans="1:12" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="40" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B42" s="40"/>
       <c r="C42" s="40"/>
@@ -6580,7 +6580,7 @@
     </row>
     <row r="43" spans="1:12" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="40" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B43" s="40"/>
       <c r="C43" s="40"/>
@@ -6596,7 +6596,7 @@
     </row>
     <row r="44" spans="1:12" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="40" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B44" s="40"/>
       <c r="C44" s="40"/>
@@ -6610,7 +6610,7 @@
     </row>
     <row r="45" spans="1:12" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="40" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B45" s="40"/>
       <c r="C45" s="40"/>
@@ -6622,12 +6622,12 @@
     </row>
     <row r="47" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A47" s="34" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="94.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="39" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B48" s="39"/>
       <c r="C48" s="39"/>
@@ -7347,10 +7347,10 @@
         <v>0</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E17" s="1">
         <v>138</v>
@@ -7387,10 +7387,10 @@
         <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E18" s="1">
         <v>189</v>
@@ -7427,10 +7427,10 @@
         <v>2</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E19" s="1">
         <v>152</v>
@@ -7467,10 +7467,10 @@
         <v>0</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E20" s="1">
         <v>113</v>
@@ -7506,10 +7506,10 @@
         <v>1</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E21" s="1">
         <v>197</v>
@@ -7545,10 +7545,10 @@
         <v>2</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E22" s="1">
         <v>107</v>
@@ -7856,7 +7856,7 @@
       <c r="Z2" s="48"/>
       <c r="AA2" s="48"/>
       <c r="AC2" s="39" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="AD2" s="39"/>
       <c r="AE2" s="39"/>
@@ -10363,7 +10363,7 @@
   </sheetData>
   <phoneticPr fontId="9" type="noConversion"/>
   <conditionalFormatting sqref="A2:G10">
-    <cfRule type="expression" dxfId="12" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2="Best"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11074,7 +11074,7 @@
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="57" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B23" s="57"/>
       <c r="C23" s="57"/>
@@ -11140,7 +11140,7 @@
     </row>
     <row r="3" spans="1:12" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="141" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B3" s="141"/>
       <c r="C3" s="141"/>
@@ -11670,7 +11670,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="88" t="s">
-        <v>97</v>
+        <v>147</v>
       </c>
       <c r="B47" s="89"/>
       <c r="C47" s="89"/>
@@ -11700,7 +11700,7 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="91" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B50" s="92"/>
       <c r="C50" s="92"/>
@@ -11744,14 +11744,14 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="77" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B53" s="74"/>
       <c r="C53" s="74"/>
       <c r="D53" s="74"/>
       <c r="E53" s="74"/>
       <c r="F53" s="74" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G53" s="74"/>
       <c r="H53" s="74"/>
@@ -11762,14 +11762,14 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54" s="64" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B54" s="65"/>
       <c r="C54" s="65"/>
       <c r="D54" s="65"/>
       <c r="E54" s="65"/>
       <c r="F54" s="65" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G54" s="65"/>
       <c r="H54" s="65"/>
@@ -11841,7 +11841,7 @@
       <c r="D58" s="65"/>
       <c r="E58" s="65"/>
       <c r="F58" s="65" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G58" s="65"/>
       <c r="H58" s="65"/>
@@ -11859,7 +11859,7 @@
       <c r="D59" s="67"/>
       <c r="E59" s="67"/>
       <c r="F59" s="67" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G59" s="67"/>
       <c r="H59" s="67"/>
@@ -11870,14 +11870,14 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="68" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B60" s="69"/>
       <c r="C60" s="69"/>
       <c r="D60" s="69"/>
       <c r="E60" s="69"/>
       <c r="F60" s="69" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G60" s="69"/>
       <c r="H60" s="69"/>
@@ -11888,7 +11888,7 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61" s="58" t="s">
-        <v>106</v>
+        <v>148</v>
       </c>
       <c r="B61" s="59"/>
       <c r="C61" s="59"/>
@@ -11974,7 +11974,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="52" orientation="landscape" horizontalDpi="90" verticalDpi="90" r:id="rId1"/>
+  <pageSetup scale="49" orientation="landscape" horizontalDpi="90" verticalDpi="90" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>

</xml_diff>